<commit_message>
- Errores avanzados (falta hora de vuelos y todo lo de comidas)
</commit_message>
<xml_diff>
--- a/Carga_Diego.xlsx
+++ b/Carga_Diego.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16885" uniqueCount="2067">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17039" uniqueCount="2067">
   <si>
     <t xml:space="preserve">Activo</t>
   </si>
@@ -6800,10 +6800,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -6821,6 +6817,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -16608,7 +16608,7 @@
       <c r="CU37" s="39"/>
       <c r="CV37" s="38"/>
     </row>
-    <row r="38" s="47" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" s="47" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="41" t="s">
         <v>106</v>
       </c>
@@ -16769,9 +16769,7 @@
       <c r="BD38" s="39"/>
       <c r="BE38" s="39"/>
       <c r="BF38" s="38"/>
-      <c r="BG38" s="38" t="s">
-        <v>358</v>
-      </c>
+      <c r="BG38" s="0"/>
       <c r="BH38" s="46" t="s">
         <v>128</v>
       </c>
@@ -17606,7 +17604,7 @@
       <c r="CU41" s="67"/>
       <c r="CV41" s="66"/>
     </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="41" t="s">
         <v>106</v>
       </c>
@@ -17763,9 +17761,7 @@
       <c r="BD42" s="39"/>
       <c r="BE42" s="39"/>
       <c r="BF42" s="66"/>
-      <c r="BG42" s="66" t="s">
-        <v>358</v>
-      </c>
+      <c r="BG42" s="0"/>
       <c r="BH42" s="46" t="s">
         <v>128</v>
       </c>
@@ -18021,8 +18017,12 @@
       <c r="BE43" s="39" t="n">
         <v>45614</v>
       </c>
-      <c r="BF43" s="66"/>
-      <c r="BG43" s="38"/>
+      <c r="BF43" s="66" t="s">
+        <v>165</v>
+      </c>
+      <c r="BG43" s="66" t="s">
+        <v>358</v>
+      </c>
       <c r="BH43" s="46" t="s">
         <v>128</v>
       </c>
@@ -18768,7 +18768,9 @@
       <c r="BE46" s="39" t="n">
         <v>45613</v>
       </c>
-      <c r="BF46" s="66"/>
+      <c r="BF46" s="66" t="s">
+        <v>357</v>
+      </c>
       <c r="BG46" s="66" t="s">
         <v>358</v>
       </c>
@@ -19035,7 +19037,9 @@
       <c r="BE47" s="39" t="n">
         <v>45613</v>
       </c>
-      <c r="BF47" s="66"/>
+      <c r="BF47" s="66" t="s">
+        <v>357</v>
+      </c>
       <c r="BG47" s="66" t="s">
         <v>358</v>
       </c>
@@ -21444,6 +21448,9 @@
       </c>
       <c r="BE57" s="39" t="n">
         <v>45613</v>
+      </c>
+      <c r="BF57" s="1" t="s">
+        <v>357</v>
       </c>
       <c r="BG57" s="1" t="s">
         <v>358</v>
@@ -32765,9 +32772,15 @@
       <c r="AX109" s="41" t="s">
         <v>139</v>
       </c>
-      <c r="AY109" s="64"/>
-      <c r="AZ109" s="64"/>
-      <c r="BA109" s="41"/>
+      <c r="AY109" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AZ109" s="5" t="n">
+        <v>45649</v>
+      </c>
+      <c r="BA109" s="41" t="s">
+        <v>357</v>
+      </c>
       <c r="BB109" s="41" t="s">
         <v>357</v>
       </c>
@@ -32971,9 +32984,15 @@
       <c r="AX110" s="41" t="s">
         <v>139</v>
       </c>
-      <c r="AY110" s="64"/>
-      <c r="AZ110" s="64"/>
-      <c r="BA110" s="41"/>
+      <c r="AY110" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AZ110" s="5" t="n">
+        <v>45649</v>
+      </c>
+      <c r="BA110" s="41" t="s">
+        <v>357</v>
+      </c>
       <c r="BB110" s="41" t="s">
         <v>357</v>
       </c>
@@ -33373,8 +33392,12 @@
       </c>
       <c r="AY112" s="64"/>
       <c r="AZ112" s="64"/>
-      <c r="BA112" s="41"/>
-      <c r="BB112" s="41"/>
+      <c r="BA112" s="41" t="s">
+        <v>357</v>
+      </c>
+      <c r="BB112" s="41" t="s">
+        <v>357</v>
+      </c>
       <c r="BC112" s="38" t="s">
         <v>128</v>
       </c>
@@ -33554,7 +33577,9 @@
       <c r="AY113" s="64"/>
       <c r="AZ113" s="64"/>
       <c r="BA113" s="41"/>
-      <c r="BB113" s="41"/>
+      <c r="BB113" s="41" t="s">
+        <v>357</v>
+      </c>
       <c r="BC113" s="38" t="s">
         <v>128</v>
       </c>
@@ -42087,6 +42112,9 @@
       <c r="BA148" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB148" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC148" s="1" t="s">
         <v>950</v>
       </c>
@@ -42099,7 +42127,9 @@
       <c r="BF148" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG148" s="38"/>
+      <c r="BG148" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH148" s="46" t="s">
         <v>128</v>
       </c>
@@ -42321,6 +42351,9 @@
       <c r="BA149" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB149" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC149" s="1" t="s">
         <v>950</v>
       </c>
@@ -42333,7 +42366,9 @@
       <c r="BF149" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG149" s="38"/>
+      <c r="BG149" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH149" s="46" t="s">
         <v>128</v>
       </c>
@@ -42561,6 +42596,9 @@
       <c r="BA150" s="1" t="s">
         <v>165</v>
       </c>
+      <c r="BB150" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC150" s="1" t="s">
         <v>950</v>
       </c>
@@ -42573,7 +42611,9 @@
       <c r="BF150" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="BG150" s="38"/>
+      <c r="BG150" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH150" s="46" t="s">
         <v>128</v>
       </c>
@@ -42801,6 +42841,9 @@
       <c r="BA151" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB151" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC151" s="1" t="s">
         <v>950</v>
       </c>
@@ -42813,7 +42856,9 @@
       <c r="BF151" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG151" s="38"/>
+      <c r="BG151" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH151" s="46" t="s">
         <v>128</v>
       </c>
@@ -43035,6 +43080,9 @@
       <c r="BA152" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB152" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC152" s="1" t="s">
         <v>950</v>
       </c>
@@ -43047,7 +43095,9 @@
       <c r="BF152" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG152" s="38"/>
+      <c r="BG152" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH152" s="46" t="s">
         <v>128</v>
       </c>
@@ -43269,6 +43319,9 @@
       <c r="BA153" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB153" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC153" s="1" t="s">
         <v>950</v>
       </c>
@@ -43281,7 +43334,9 @@
       <c r="BF153" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG153" s="38"/>
+      <c r="BG153" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH153" s="46" t="s">
         <v>128</v>
       </c>
@@ -43503,6 +43558,9 @@
       <c r="BA154" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB154" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC154" s="1" t="s">
         <v>950</v>
       </c>
@@ -43515,7 +43573,9 @@
       <c r="BF154" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG154" s="38"/>
+      <c r="BG154" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH154" s="46" t="s">
         <v>128</v>
       </c>
@@ -43737,6 +43797,9 @@
       <c r="BA155" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB155" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC155" s="1" t="s">
         <v>950</v>
       </c>
@@ -43749,7 +43812,9 @@
       <c r="BF155" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG155" s="38"/>
+      <c r="BG155" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH155" s="46" t="s">
         <v>128</v>
       </c>
@@ -43977,6 +44042,9 @@
       <c r="BA156" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB156" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC156" s="1" t="s">
         <v>950</v>
       </c>
@@ -43989,7 +44057,9 @@
       <c r="BF156" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG156" s="38"/>
+      <c r="BG156" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH156" s="46" t="s">
         <v>128</v>
       </c>
@@ -44217,6 +44287,9 @@
       <c r="BA157" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB157" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC157" s="1" t="s">
         <v>950</v>
       </c>
@@ -44229,7 +44302,9 @@
       <c r="BF157" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG157" s="38"/>
+      <c r="BG157" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH157" s="46" t="s">
         <v>128</v>
       </c>
@@ -44457,6 +44532,9 @@
       <c r="BA158" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB158" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC158" s="1" t="s">
         <v>950</v>
       </c>
@@ -44469,7 +44547,9 @@
       <c r="BF158" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG158" s="38"/>
+      <c r="BG158" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH158" s="46" t="s">
         <v>128</v>
       </c>
@@ -44697,6 +44777,9 @@
       <c r="BA159" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB159" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC159" s="1" t="s">
         <v>950</v>
       </c>
@@ -44709,7 +44792,9 @@
       <c r="BF159" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG159" s="38"/>
+      <c r="BG159" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH159" s="46" t="s">
         <v>128</v>
       </c>
@@ -44937,6 +45022,9 @@
       <c r="BA160" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB160" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC160" s="1" t="s">
         <v>950</v>
       </c>
@@ -44949,7 +45037,9 @@
       <c r="BF160" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG160" s="38"/>
+      <c r="BG160" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH160" s="46" t="s">
         <v>128</v>
       </c>
@@ -45177,6 +45267,9 @@
       <c r="BA161" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB161" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC161" s="1" t="s">
         <v>950</v>
       </c>
@@ -45189,7 +45282,9 @@
       <c r="BF161" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG161" s="38"/>
+      <c r="BG161" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH161" s="46" t="s">
         <v>128</v>
       </c>
@@ -45417,6 +45512,9 @@
       <c r="BA162" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB162" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC162" s="1" t="s">
         <v>950</v>
       </c>
@@ -45429,7 +45527,9 @@
       <c r="BF162" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG162" s="38"/>
+      <c r="BG162" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH162" s="46" t="s">
         <v>128</v>
       </c>
@@ -45657,6 +45757,9 @@
       <c r="BA163" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB163" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC163" s="1" t="s">
         <v>950</v>
       </c>
@@ -45669,7 +45772,9 @@
       <c r="BF163" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG163" s="38"/>
+      <c r="BG163" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH163" s="46" t="s">
         <v>128</v>
       </c>
@@ -45897,6 +46002,9 @@
       <c r="BA164" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB164" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC164" s="1" t="s">
         <v>950</v>
       </c>
@@ -45909,7 +46017,9 @@
       <c r="BF164" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG164" s="38"/>
+      <c r="BG164" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH164" s="46" t="s">
         <v>128</v>
       </c>
@@ -46137,6 +46247,9 @@
       <c r="BA165" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB165" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC165" s="1" t="s">
         <v>950</v>
       </c>
@@ -46149,7 +46262,9 @@
       <c r="BF165" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG165" s="38"/>
+      <c r="BG165" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH165" s="46" t="s">
         <v>128</v>
       </c>
@@ -46377,6 +46492,9 @@
       <c r="BA166" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB166" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC166" s="1" t="s">
         <v>950</v>
       </c>
@@ -46389,7 +46507,9 @@
       <c r="BF166" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG166" s="38"/>
+      <c r="BG166" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH166" s="46" t="s">
         <v>128</v>
       </c>
@@ -46617,6 +46737,9 @@
       <c r="BA167" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB167" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC167" s="1" t="s">
         <v>950</v>
       </c>
@@ -46629,7 +46752,9 @@
       <c r="BF167" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG167" s="38"/>
+      <c r="BG167" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH167" s="46" t="s">
         <v>128</v>
       </c>
@@ -46857,6 +46982,9 @@
       <c r="BA168" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB168" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC168" s="1" t="s">
         <v>950</v>
       </c>
@@ -46869,7 +46997,9 @@
       <c r="BF168" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG168" s="38"/>
+      <c r="BG168" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH168" s="46" t="s">
         <v>128</v>
       </c>
@@ -47097,6 +47227,9 @@
       <c r="BA169" s="1" t="s">
         <v>165</v>
       </c>
+      <c r="BB169" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="BC169" s="1" t="s">
         <v>950</v>
       </c>
@@ -47109,7 +47242,9 @@
       <c r="BF169" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="BG169" s="38"/>
+      <c r="BG169" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH169" s="46" t="s">
         <v>128</v>
       </c>
@@ -47297,6 +47432,9 @@
       </c>
       <c r="BA170" s="1" t="s">
         <v>165</v>
+      </c>
+      <c r="BB170" s="1" t="s">
+        <v>141</v>
       </c>
       <c r="BC170" s="38" t="s">
         <v>128</v>
@@ -47945,6 +48083,9 @@
       <c r="BA174" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB174" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC174" s="1" t="s">
         <v>950</v>
       </c>
@@ -47957,7 +48098,9 @@
       <c r="BF174" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BG174" s="38"/>
+      <c r="BG174" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH174" s="46" t="s">
         <v>128</v>
       </c>
@@ -48182,6 +48325,9 @@
       <c r="BA175" s="1" t="s">
         <v>165</v>
       </c>
+      <c r="BB175" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC175" s="1" t="s">
         <v>950</v>
       </c>
@@ -48194,7 +48340,9 @@
       <c r="BF175" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="BG175" s="38"/>
+      <c r="BG175" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH175" s="46" t="s">
         <v>128</v>
       </c>
@@ -48413,6 +48561,9 @@
       <c r="BA176" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB176" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC176" s="1" t="s">
         <v>950</v>
       </c>
@@ -48425,7 +48576,9 @@
       <c r="BF176" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BG176" s="38"/>
+      <c r="BG176" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH176" s="46" t="s">
         <v>128</v>
       </c>
@@ -48644,6 +48797,9 @@
       <c r="BA177" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB177" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC177" s="1" t="s">
         <v>950</v>
       </c>
@@ -48656,7 +48812,9 @@
       <c r="BF177" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BG177" s="38"/>
+      <c r="BG177" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH177" s="46" t="s">
         <v>128</v>
       </c>
@@ -48875,6 +49033,9 @@
       <c r="BA178" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB178" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC178" s="1" t="s">
         <v>950</v>
       </c>
@@ -48887,7 +49048,9 @@
       <c r="BF178" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BG178" s="38"/>
+      <c r="BG178" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH178" s="46" t="s">
         <v>128</v>
       </c>
@@ -49100,6 +49263,9 @@
       <c r="BA179" s="1" t="s">
         <v>165</v>
       </c>
+      <c r="BB179" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC179" s="1" t="s">
         <v>950</v>
       </c>
@@ -49112,7 +49278,9 @@
       <c r="BF179" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="BG179" s="38"/>
+      <c r="BG179" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH179" s="46" t="s">
         <v>128</v>
       </c>
@@ -49325,6 +49493,9 @@
       <c r="BA180" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB180" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC180" s="1" t="s">
         <v>950</v>
       </c>
@@ -49337,7 +49508,9 @@
       <c r="BF180" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BG180" s="38"/>
+      <c r="BG180" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH180" s="46" t="s">
         <v>128</v>
       </c>
@@ -49550,6 +49723,9 @@
       <c r="BA181" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB181" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC181" s="1" t="s">
         <v>950</v>
       </c>
@@ -49562,7 +49738,9 @@
       <c r="BF181" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BG181" s="38"/>
+      <c r="BG181" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH181" s="46" t="s">
         <v>128</v>
       </c>
@@ -49775,6 +49953,9 @@
       <c r="BA182" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB182" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC182" s="1" t="s">
         <v>950</v>
       </c>
@@ -49787,7 +49968,9 @@
       <c r="BF182" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BG182" s="38"/>
+      <c r="BG182" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH182" s="46" t="s">
         <v>128</v>
       </c>
@@ -50006,6 +50189,9 @@
       <c r="BA183" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB183" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC183" s="1" t="s">
         <v>950</v>
       </c>
@@ -50018,7 +50204,9 @@
       <c r="BF183" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BG183" s="38"/>
+      <c r="BG183" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH183" s="46" t="s">
         <v>128</v>
       </c>
@@ -50204,6 +50392,12 @@
       <c r="AX184" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY184" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AZ184" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BA184" s="1" t="s">
         <v>140</v>
       </c>
@@ -50222,7 +50416,9 @@
       <c r="BF184" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BG184" s="38"/>
+      <c r="BG184" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH184" s="1" t="s">
         <v>357</v>
       </c>
@@ -50441,6 +50637,9 @@
       <c r="BA185" s="1" t="s">
         <v>165</v>
       </c>
+      <c r="BB185" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC185" s="1" t="s">
         <v>950</v>
       </c>
@@ -50453,7 +50652,9 @@
       <c r="BF185" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="BG185" s="38"/>
+      <c r="BG185" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH185" s="46" t="s">
         <v>128</v>
       </c>
@@ -50639,6 +50840,12 @@
       <c r="AX186" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY186" s="5" t="n">
+        <v>45629</v>
+      </c>
+      <c r="AZ186" s="5" t="n">
+        <v>45630</v>
+      </c>
       <c r="BA186" s="1" t="s">
         <v>165</v>
       </c>
@@ -50657,7 +50864,9 @@
       <c r="BF186" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="BG186" s="38"/>
+      <c r="BG186" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH186" s="1" t="s">
         <v>357</v>
       </c>
@@ -50867,18 +51076,33 @@
       <c r="AX187" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY187" s="5" t="n">
+        <v>45630</v>
+      </c>
+      <c r="AZ187" s="5" t="n">
+        <v>45631</v>
+      </c>
       <c r="BA187" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB187" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC187" s="1" t="s">
         <v>950</v>
       </c>
-      <c r="BD187" s="5"/>
-      <c r="BE187" s="5"/>
+      <c r="BD187" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE187" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF187" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BG187" s="38"/>
+      <c r="BG187" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH187" s="46" t="s">
         <v>128</v>
       </c>
@@ -51073,16 +51297,33 @@
       <c r="AX188" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY188" s="5" t="n">
+        <v>45631</v>
+      </c>
+      <c r="AZ188" s="5" t="n">
+        <v>45632</v>
+      </c>
       <c r="BA188" s="1" t="s">
         <v>165</v>
       </c>
+      <c r="BB188" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC188" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD188" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE188" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF188" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="BG188" s="38"/>
+      <c r="BG188" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH188" s="46" t="s">
         <v>128</v>
       </c>
@@ -51298,16 +51539,33 @@
       <c r="AX189" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY189" s="5" t="n">
+        <v>45632</v>
+      </c>
+      <c r="AZ189" s="5" t="n">
+        <v>45633</v>
+      </c>
       <c r="BA189" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB189" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC189" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD189" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE189" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF189" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG189" s="38"/>
+      <c r="BG189" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH189" s="46" t="s">
         <v>128</v>
       </c>
@@ -51517,16 +51775,33 @@
       <c r="AX190" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY190" s="5" t="n">
+        <v>45633</v>
+      </c>
+      <c r="AZ190" s="5" t="n">
+        <v>45634</v>
+      </c>
       <c r="BA190" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB190" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC190" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD190" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE190" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF190" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG190" s="38"/>
+      <c r="BG190" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH190" s="46" t="s">
         <v>128</v>
       </c>
@@ -51736,16 +52011,33 @@
       <c r="AX191" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY191" s="5" t="n">
+        <v>45634</v>
+      </c>
+      <c r="AZ191" s="5" t="n">
+        <v>45635</v>
+      </c>
       <c r="BA191" s="1" t="s">
         <v>165</v>
       </c>
+      <c r="BB191" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC191" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD191" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE191" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF191" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="BG191" s="38"/>
+      <c r="BG191" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH191" s="46" t="s">
         <v>128</v>
       </c>
@@ -51955,16 +52247,33 @@
       <c r="AX192" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY192" s="5" t="n">
+        <v>45635</v>
+      </c>
+      <c r="AZ192" s="5" t="n">
+        <v>45636</v>
+      </c>
       <c r="BA192" s="1" t="s">
         <v>165</v>
       </c>
+      <c r="BB192" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC192" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD192" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE192" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF192" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="BG192" s="38"/>
+      <c r="BG192" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH192" s="46" t="s">
         <v>128</v>
       </c>
@@ -52174,16 +52483,33 @@
       <c r="AX193" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY193" s="5" t="n">
+        <v>45636</v>
+      </c>
+      <c r="AZ193" s="5" t="n">
+        <v>45637</v>
+      </c>
       <c r="BA193" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB193" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC193" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD193" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE193" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF193" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG193" s="38"/>
+      <c r="BG193" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH193" s="46" t="s">
         <v>128</v>
       </c>
@@ -52393,16 +52719,33 @@
       <c r="AX194" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY194" s="5" t="n">
+        <v>45637</v>
+      </c>
+      <c r="AZ194" s="5" t="n">
+        <v>45638</v>
+      </c>
       <c r="BA194" s="1" t="s">
         <v>165</v>
       </c>
+      <c r="BB194" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC194" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD194" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE194" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF194" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="BG194" s="38"/>
+      <c r="BG194" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH194" s="46" t="s">
         <v>128</v>
       </c>
@@ -52612,16 +52955,33 @@
       <c r="AX195" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY195" s="5" t="n">
+        <v>45638</v>
+      </c>
+      <c r="AZ195" s="5" t="n">
+        <v>45639</v>
+      </c>
       <c r="BA195" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB195" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC195" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD195" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE195" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF195" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG195" s="38"/>
+      <c r="BG195" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH195" s="46" t="s">
         <v>128</v>
       </c>
@@ -52825,16 +53185,33 @@
       <c r="AX196" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY196" s="5" t="n">
+        <v>45639</v>
+      </c>
+      <c r="AZ196" s="5" t="n">
+        <v>45640</v>
+      </c>
       <c r="BA196" s="1" t="s">
         <v>165</v>
       </c>
+      <c r="BB196" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC196" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD196" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE196" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF196" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="BG196" s="38"/>
+      <c r="BG196" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH196" s="46" t="s">
         <v>128</v>
       </c>
@@ -53050,16 +53427,33 @@
       <c r="AX197" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY197" s="5" t="n">
+        <v>45640</v>
+      </c>
+      <c r="AZ197" s="5" t="n">
+        <v>45641</v>
+      </c>
       <c r="BA197" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB197" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC197" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD197" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE197" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF197" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG197" s="38"/>
+      <c r="BG197" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH197" s="46" t="s">
         <v>128</v>
       </c>
@@ -53269,16 +53663,33 @@
       <c r="AX198" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY198" s="5" t="n">
+        <v>45641</v>
+      </c>
+      <c r="AZ198" s="5" t="n">
+        <v>45642</v>
+      </c>
       <c r="BA198" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB198" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC198" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD198" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE198" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF198" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG198" s="38"/>
+      <c r="BG198" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH198" s="46" t="s">
         <v>128</v>
       </c>
@@ -53488,16 +53899,33 @@
       <c r="AX199" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY199" s="5" t="n">
+        <v>45642</v>
+      </c>
+      <c r="AZ199" s="5" t="n">
+        <v>45643</v>
+      </c>
       <c r="BA199" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB199" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC199" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD199" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE199" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF199" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG199" s="38"/>
+      <c r="BG199" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH199" s="46" t="s">
         <v>128</v>
       </c>
@@ -53707,16 +54135,33 @@
       <c r="AX200" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY200" s="5" t="n">
+        <v>45643</v>
+      </c>
+      <c r="AZ200" s="5" t="n">
+        <v>45644</v>
+      </c>
       <c r="BA200" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB200" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC200" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD200" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE200" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF200" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG200" s="38"/>
+      <c r="BG200" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH200" s="46" t="s">
         <v>128</v>
       </c>
@@ -53926,16 +54371,33 @@
       <c r="AX201" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY201" s="5" t="n">
+        <v>45644</v>
+      </c>
+      <c r="AZ201" s="5" t="n">
+        <v>45645</v>
+      </c>
       <c r="BA201" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB201" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC201" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD201" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE201" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF201" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG201" s="38"/>
+      <c r="BG201" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH201" s="46" t="s">
         <v>128</v>
       </c>
@@ -54121,6 +54583,12 @@
       <c r="AX202" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY202" s="5" t="n">
+        <v>45645</v>
+      </c>
+      <c r="AZ202" s="5" t="n">
+        <v>45646</v>
+      </c>
       <c r="BA202" s="1" t="s">
         <v>140</v>
       </c>
@@ -54130,10 +54598,18 @@
       <c r="BC202" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD202" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE202" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF202" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG202" s="38"/>
+      <c r="BG202" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH202" s="1" t="s">
         <v>357</v>
       </c>
@@ -54337,16 +54813,33 @@
       <c r="AX203" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY203" s="5" t="n">
+        <v>45646</v>
+      </c>
+      <c r="AZ203" s="5" t="n">
+        <v>45647</v>
+      </c>
       <c r="BA203" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB203" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC203" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD203" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE203" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF203" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG203" s="38"/>
+      <c r="BG203" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH203" s="46" t="s">
         <v>128</v>
       </c>
@@ -54556,16 +55049,33 @@
       <c r="AX204" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY204" s="5" t="n">
+        <v>45647</v>
+      </c>
+      <c r="AZ204" s="5" t="n">
+        <v>45648</v>
+      </c>
       <c r="BA204" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="BB204" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC204" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD204" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE204" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF204" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="BG204" s="38"/>
+      <c r="BG204" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH204" s="46" t="s">
         <v>128</v>
       </c>
@@ -54775,16 +55285,33 @@
       <c r="AX205" s="1" t="s">
         <v>139</v>
       </c>
+      <c r="AY205" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AZ205" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BA205" s="1" t="s">
         <v>165</v>
       </c>
+      <c r="BB205" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC205" s="1" t="s">
         <v>950</v>
       </c>
+      <c r="BD205" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="BE205" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BF205" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="BG205" s="38"/>
+      <c r="BG205" s="1" t="s">
+        <v>987</v>
+      </c>
       <c r="BH205" s="46" t="s">
         <v>128</v>
       </c>
@@ -54981,6 +55508,9 @@
       </c>
       <c r="BA206" s="1" t="s">
         <v>165</v>
+      </c>
+      <c r="BB206" s="1" t="s">
+        <v>1320</v>
       </c>
       <c r="BC206" s="38" t="s">
         <v>128</v>
@@ -55155,6 +55685,9 @@
       <c r="BA207" s="1" t="s">
         <v>165</v>
       </c>
+      <c r="BB207" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC207" s="38" t="s">
         <v>128</v>
       </c>
@@ -55327,6 +55860,9 @@
       <c r="BA208" s="1" t="s">
         <v>165</v>
       </c>
+      <c r="BB208" s="1" t="s">
+        <v>1320</v>
+      </c>
       <c r="BC208" s="38" t="s">
         <v>128</v>
       </c>
@@ -55496,8 +56032,12 @@
       <c r="AX209" s="46" t="s">
         <v>139</v>
       </c>
-      <c r="AY209" s="92"/>
-      <c r="AZ209" s="92"/>
+      <c r="AY209" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AZ209" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="BA209" s="46" t="s">
         <v>165</v>
       </c>
@@ -55505,7 +56045,7 @@
         <v>106</v>
       </c>
       <c r="BC209" s="38" t="s">
-        <v>128</v>
+        <v>475</v>
       </c>
       <c r="BD209" s="39" t="n">
         <v>45610</v>
@@ -55513,7 +56053,9 @@
       <c r="BE209" s="39" t="n">
         <v>45613</v>
       </c>
-      <c r="BF209" s="38"/>
+      <c r="BF209" s="1" t="s">
+        <v>165</v>
+      </c>
       <c r="BG209" s="38" t="s">
         <v>358</v>
       </c>
@@ -55574,11 +56116,11 @@
       <c r="C210" s="46" t="s">
         <v>707</v>
       </c>
-      <c r="D210" s="93"/>
-      <c r="E210" s="94" t="n">
+      <c r="D210" s="92"/>
+      <c r="E210" s="93" t="n">
         <v>45627</v>
       </c>
-      <c r="F210" s="94" t="n">
+      <c r="F210" s="93" t="n">
         <v>45627</v>
       </c>
       <c r="G210" s="46" t="s">
@@ -55587,46 +56129,46 @@
       <c r="H210" s="46" t="s">
         <v>111</v>
       </c>
-      <c r="I210" s="95" t="s">
+      <c r="I210" s="94" t="s">
         <v>112</v>
       </c>
-      <c r="J210" s="95" t="s">
+      <c r="J210" s="94" t="s">
         <v>112</v>
       </c>
-      <c r="K210" s="96" t="s">
+      <c r="K210" s="95" t="s">
         <v>1533</v>
       </c>
-      <c r="L210" s="96" t="s">
+      <c r="L210" s="95" t="s">
         <v>1534</v>
       </c>
       <c r="M210" s="46" t="s">
         <v>151</v>
       </c>
-      <c r="N210" s="96" t="s">
+      <c r="N210" s="95" t="s">
         <v>734</v>
       </c>
-      <c r="O210" s="96" t="s">
+      <c r="O210" s="95" t="s">
         <v>920</v>
       </c>
       <c r="P210" s="46" t="s">
         <v>1535</v>
       </c>
-      <c r="Q210" s="97" t="n">
+      <c r="Q210" s="96" t="n">
         <v>28395</v>
       </c>
-      <c r="R210" s="96" t="s">
+      <c r="R210" s="95" t="s">
         <v>121</v>
       </c>
-      <c r="S210" s="96" t="s">
+      <c r="S210" s="95" t="s">
         <v>121</v>
       </c>
-      <c r="T210" s="96" t="s">
+      <c r="T210" s="95" t="s">
         <v>121</v>
       </c>
       <c r="U210" s="46"/>
-      <c r="V210" s="96"/>
-      <c r="W210" s="92"/>
-      <c r="X210" s="94"/>
+      <c r="V210" s="95"/>
+      <c r="W210" s="97"/>
+      <c r="X210" s="93"/>
       <c r="Y210" s="98" t="s">
         <v>128</v>
       </c>
@@ -55640,7 +56182,7 @@
       <c r="AE210" s="98" t="s">
         <v>1536</v>
       </c>
-      <c r="AF210" s="92"/>
+      <c r="AF210" s="97"/>
       <c r="AG210" s="46"/>
       <c r="AH210" s="100" t="s">
         <v>121</v>
@@ -55652,25 +56194,25 @@
         <v>121</v>
       </c>
       <c r="AK210" s="101"/>
-      <c r="AL210" s="94"/>
+      <c r="AL210" s="93"/>
       <c r="AM210" s="102"/>
       <c r="AN210" s="103"/>
-      <c r="AO210" s="92"/>
+      <c r="AO210" s="97"/>
       <c r="AP210" s="104"/>
-      <c r="AQ210" s="95" t="s">
+      <c r="AQ210" s="94" t="s">
         <v>134</v>
       </c>
-      <c r="AR210" s="95" t="s">
+      <c r="AR210" s="94" t="s">
         <v>135</v>
       </c>
-      <c r="AS210" s="95" t="s">
+      <c r="AS210" s="94" t="s">
         <v>136</v>
       </c>
       <c r="AT210" s="46" t="s">
         <v>137</v>
       </c>
-      <c r="AU210" s="95"/>
-      <c r="AV210" s="95"/>
+      <c r="AU210" s="94"/>
+      <c r="AV210" s="94"/>
       <c r="AW210" s="105" t="n">
         <v>80</v>
       </c>
@@ -55707,8 +56249,8 @@
       <c r="BH210" s="46" t="s">
         <v>128</v>
       </c>
-      <c r="BI210" s="93"/>
-      <c r="BJ210" s="93"/>
+      <c r="BI210" s="92"/>
+      <c r="BJ210" s="92"/>
       <c r="BK210" s="46"/>
       <c r="BL210" s="46"/>
       <c r="BM210" s="46" t="s">
@@ -55717,7 +56259,7 @@
       <c r="BN210" s="46"/>
       <c r="BO210" s="46"/>
       <c r="BP210" s="46"/>
-      <c r="BQ210" s="92"/>
+      <c r="BQ210" s="97"/>
       <c r="BR210" s="106"/>
       <c r="BS210" s="41" t="s">
         <v>128</v>
@@ -55745,8 +56287,8 @@
       <c r="CJ210" s="107"/>
       <c r="CK210" s="46"/>
       <c r="CL210" s="46"/>
-      <c r="CM210" s="92"/>
-      <c r="CN210" s="92"/>
+      <c r="CM210" s="97"/>
+      <c r="CN210" s="97"/>
       <c r="CO210" s="46"/>
       <c r="CP210" s="46"/>
       <c r="CQ210" s="46"/>
@@ -61905,8 +62447,17 @@
       <c r="AL26" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM26" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN26" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AO26" s="10" t="s">
         <v>140</v>
+      </c>
+      <c r="AP26" s="10" t="s">
+        <v>987</v>
       </c>
       <c r="AQ26" s="10" t="s">
         <v>128</v>
@@ -62086,8 +62637,17 @@
       <c r="AL27" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM27" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN27" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AO27" s="10" t="s">
         <v>140</v>
+      </c>
+      <c r="AP27" s="10" t="s">
+        <v>987</v>
       </c>
       <c r="AQ27" s="10" t="s">
         <v>128</v>
@@ -62267,8 +62827,17 @@
       <c r="AL28" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM28" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN28" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AO28" s="10" t="s">
         <v>140</v>
+      </c>
+      <c r="AP28" s="10" t="s">
+        <v>987</v>
       </c>
       <c r="AQ28" s="10" t="s">
         <v>128</v>
@@ -62448,8 +63017,17 @@
       <c r="AL29" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM29" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN29" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AO29" s="10" t="s">
         <v>140</v>
+      </c>
+      <c r="AP29" s="10" t="s">
+        <v>987</v>
       </c>
       <c r="AQ29" s="10" t="s">
         <v>128</v>
@@ -62629,8 +63207,17 @@
       <c r="AL30" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM30" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN30" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AO30" s="10" t="s">
         <v>140</v>
+      </c>
+      <c r="AP30" s="10" t="s">
+        <v>987</v>
       </c>
       <c r="AQ30" s="10" t="s">
         <v>128</v>
@@ -62810,8 +63397,17 @@
       <c r="AL31" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM31" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN31" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AO31" s="10" t="s">
         <v>140</v>
+      </c>
+      <c r="AP31" s="10" t="s">
+        <v>987</v>
       </c>
       <c r="AQ31" s="10" t="s">
         <v>128</v>
@@ -62991,8 +63587,17 @@
       <c r="AL32" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM32" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN32" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AO32" s="10" t="s">
         <v>140</v>
+      </c>
+      <c r="AP32" s="10" t="s">
+        <v>987</v>
       </c>
       <c r="AQ32" s="10" t="s">
         <v>128</v>
@@ -63172,8 +63777,17 @@
       <c r="AL33" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM33" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN33" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AO33" s="10" t="s">
         <v>140</v>
+      </c>
+      <c r="AP33" s="10" t="s">
+        <v>987</v>
       </c>
       <c r="AQ33" s="10" t="s">
         <v>128</v>
@@ -63353,8 +63967,17 @@
       <c r="AL34" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM34" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN34" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AO34" s="10" t="s">
         <v>140</v>
+      </c>
+      <c r="AP34" s="10" t="s">
+        <v>987</v>
       </c>
       <c r="AQ34" s="10" t="s">
         <v>128</v>
@@ -63534,8 +64157,17 @@
       <c r="AL35" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM35" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN35" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AO35" s="10" t="s">
         <v>140</v>
+      </c>
+      <c r="AP35" s="10" t="s">
+        <v>987</v>
       </c>
       <c r="AQ35" s="10" t="s">
         <v>128</v>
@@ -63715,8 +64347,17 @@
       <c r="AL36" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM36" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN36" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AO36" s="10" t="s">
         <v>140</v>
+      </c>
+      <c r="AP36" s="10" t="s">
+        <v>987</v>
       </c>
       <c r="AQ36" s="10" t="s">
         <v>128</v>
@@ -63896,8 +64537,17 @@
       <c r="AL37" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM37" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN37" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AO37" s="10" t="s">
         <v>165</v>
+      </c>
+      <c r="AP37" s="10" t="s">
+        <v>987</v>
       </c>
       <c r="AQ37" s="10" t="s">
         <v>128</v>
@@ -64077,8 +64727,17 @@
       <c r="AL38" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM38" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN38" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AO38" s="10" t="s">
         <v>165</v>
+      </c>
+      <c r="AP38" s="10" t="s">
+        <v>987</v>
       </c>
       <c r="AQ38" s="10" t="s">
         <v>128</v>
@@ -64258,8 +64917,17 @@
       <c r="AL39" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM39" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN39" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AO39" s="10" t="s">
         <v>140</v>
+      </c>
+      <c r="AP39" s="10" t="s">
+        <v>987</v>
       </c>
       <c r="AQ39" s="10" t="s">
         <v>128</v>
@@ -64439,8 +65107,17 @@
       <c r="AL40" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM40" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN40" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AO40" s="10" t="s">
         <v>140</v>
+      </c>
+      <c r="AP40" s="10" t="s">
+        <v>987</v>
       </c>
       <c r="AQ40" s="10" t="s">
         <v>128</v>
@@ -64618,6 +65295,12 @@
       <c r="AL41" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM41" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN41" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AQ41" s="10" t="s">
         <v>128</v>
       </c>
@@ -64796,6 +65479,12 @@
       <c r="AL42" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM42" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN42" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AQ42" s="10" t="s">
         <v>128</v>
       </c>
@@ -66153,6 +66842,9 @@
         <v>939</v>
       </c>
       <c r="AN50" s="5"/>
+      <c r="AP50" s="10" t="s">
+        <v>357</v>
+      </c>
       <c r="AQ50" s="10" t="s">
         <v>128</v>
       </c>
@@ -73904,6 +74596,12 @@
       <c r="AL100" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM100" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN100" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AQ100" s="10" t="s">
         <v>128</v>
       </c>
@@ -75781,6 +76479,9 @@
       <c r="AO110" s="10" t="s">
         <v>140</v>
       </c>
+      <c r="AP110" s="10" t="s">
+        <v>141</v>
+      </c>
       <c r="AQ110" s="10" t="s">
         <v>128</v>
       </c>
@@ -75966,6 +76667,9 @@
       <c r="AO111" s="10" t="s">
         <v>140</v>
       </c>
+      <c r="AP111" s="10" t="s">
+        <v>141</v>
+      </c>
       <c r="AQ111" s="10" t="s">
         <v>128</v>
       </c>
@@ -76151,6 +76855,9 @@
       <c r="AO112" s="10" t="s">
         <v>140</v>
       </c>
+      <c r="AP112" s="10" t="s">
+        <v>141</v>
+      </c>
       <c r="AQ112" s="10" t="s">
         <v>128</v>
       </c>
@@ -76336,6 +77043,9 @@
       <c r="AO113" s="10" t="s">
         <v>140</v>
       </c>
+      <c r="AP113" s="10" t="s">
+        <v>141</v>
+      </c>
       <c r="AQ113" s="10" t="s">
         <v>128</v>
       </c>
@@ -76521,6 +77231,9 @@
       <c r="AO114" s="10" t="s">
         <v>165</v>
       </c>
+      <c r="AP114" s="10" t="s">
+        <v>141</v>
+      </c>
       <c r="AQ114" s="10" t="s">
         <v>128</v>
       </c>
@@ -76706,6 +77419,9 @@
       <c r="AO115" s="10" t="s">
         <v>140</v>
       </c>
+      <c r="AP115" s="10" t="s">
+        <v>141</v>
+      </c>
       <c r="AQ115" s="10" t="s">
         <v>128</v>
       </c>
@@ -76891,6 +77607,9 @@
       <c r="AO116" s="10" t="s">
         <v>140</v>
       </c>
+      <c r="AP116" s="10" t="s">
+        <v>141</v>
+      </c>
       <c r="AQ116" s="10" t="s">
         <v>128</v>
       </c>
@@ -77076,6 +77795,9 @@
       <c r="AO117" s="10" t="s">
         <v>140</v>
       </c>
+      <c r="AP117" s="10" t="s">
+        <v>141</v>
+      </c>
       <c r="AQ117" s="10" t="s">
         <v>128</v>
       </c>
@@ -77261,6 +77983,9 @@
       <c r="AO118" s="10" t="s">
         <v>140</v>
       </c>
+      <c r="AP118" s="10" t="s">
+        <v>141</v>
+      </c>
       <c r="AQ118" s="10" t="s">
         <v>128</v>
       </c>
@@ -77446,6 +78171,9 @@
       <c r="AO119" s="10" t="s">
         <v>140</v>
       </c>
+      <c r="AP119" s="10" t="s">
+        <v>141</v>
+      </c>
       <c r="AQ119" s="10" t="s">
         <v>128</v>
       </c>
@@ -77631,6 +78359,9 @@
       <c r="AO120" s="10" t="s">
         <v>140</v>
       </c>
+      <c r="AP120" s="10" t="s">
+        <v>141</v>
+      </c>
       <c r="AQ120" s="10" t="s">
         <v>128</v>
       </c>
@@ -77816,6 +78547,9 @@
       <c r="AO121" s="10" t="s">
         <v>140</v>
       </c>
+      <c r="AP121" s="10" t="s">
+        <v>141</v>
+      </c>
       <c r="AQ121" s="10" t="s">
         <v>128</v>
       </c>
@@ -78001,6 +78735,9 @@
       <c r="AO122" s="10" t="s">
         <v>140</v>
       </c>
+      <c r="AP122" s="10" t="s">
+        <v>141</v>
+      </c>
       <c r="AQ122" s="10" t="s">
         <v>128</v>
       </c>
@@ -78186,6 +78923,9 @@
       <c r="AO123" s="10" t="s">
         <v>140</v>
       </c>
+      <c r="AP123" s="10" t="s">
+        <v>141</v>
+      </c>
       <c r="AQ123" s="10" t="s">
         <v>128</v>
       </c>
@@ -78368,6 +79108,9 @@
       <c r="AO124" s="10" t="s">
         <v>165</v>
       </c>
+      <c r="AP124" s="10" t="s">
+        <v>141</v>
+      </c>
       <c r="AQ124" s="10" t="s">
         <v>128</v>
       </c>
@@ -78529,8 +79272,17 @@
       <c r="AL125" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM125" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN125" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AO125" s="10" t="s">
         <v>140</v>
+      </c>
+      <c r="AP125" s="10" t="s">
+        <v>141</v>
       </c>
       <c r="AQ125" s="10" t="s">
         <v>128</v>
@@ -78708,8 +79460,17 @@
       <c r="AL126" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="AM126" s="5" t="n">
+        <v>45648</v>
+      </c>
+      <c r="AN126" s="5" t="n">
+        <v>45649</v>
+      </c>
       <c r="AO126" s="10" t="s">
         <v>140</v>
+      </c>
+      <c r="AP126" s="10" t="s">
+        <v>141</v>
       </c>
       <c r="AQ126" s="10" t="s">
         <v>128</v>
@@ -78896,6 +79657,9 @@
       <c r="AO127" s="10" t="s">
         <v>140</v>
       </c>
+      <c r="AP127" s="10" t="s">
+        <v>141</v>
+      </c>
       <c r="AQ127" s="10" t="s">
         <v>128</v>
       </c>
@@ -79081,6 +79845,9 @@
       <c r="AO128" s="10" t="s">
         <v>140</v>
       </c>
+      <c r="AP128" s="10" t="s">
+        <v>141</v>
+      </c>
       <c r="AQ128" s="10" t="s">
         <v>475</v>
       </c>
@@ -79274,6 +80041,9 @@
       </c>
       <c r="AO129" s="10" t="s">
         <v>140</v>
+      </c>
+      <c r="AP129" s="10" t="s">
+        <v>141</v>
       </c>
       <c r="AQ129" s="10" t="s">
         <v>128</v>

</xml_diff>